<commit_message>
docs: record production acceptance and independent interface review
</commit_message>
<xml_diff>
--- a/docs/structured-protocol/20261014/evidence/experiment.xlsx
+++ b/docs/structured-protocol/20261014/evidence/experiment.xlsx
@@ -76,13 +76,13 @@
     <t>tags</t>
   </si>
   <si>
-    <t>合成体系验收 b9e2edc6-3b62-4995-b77d-4c0d11eccccd</t>
-  </si>
-  <si>
-    <t>SYN-b9e2edc6-3b62-4995-b77d-4c0d11eccccd</t>
-  </si>
-  <si>
-    <t>EXP-025</t>
+    <t>合成体系验收 79b5ab5c-dbd4-464b-a250-d996a01b0b48</t>
+  </si>
+  <si>
+    <t>SYN-79b5ab5c-dbd4-464b-a250-d996a01b0b48</t>
+  </si>
+  <si>
+    <t>EXP-056</t>
   </si>
   <si>
     <t>合成验收 · 页面创建与执行</t>
@@ -106,9 +106,9 @@
     <t>350／600 µL 合成规程 · 1.0</t>
   </si>
   <si>
-    <t>本次执行记录 · 当前实验组 · 源版本 350／600 µL 合成规程 v1.0（cmv7g3ccr0007w6os2aa9gaf3）
+    <t>本次执行记录 · 当前实验组 · 源版本 350／600 µL 合成规程 v1.0（cmv7gz2j200078fosfu1bvjzs）
 裂解体积：350 µL；样本性质：普通样本
-采用确认时间：2026-10-14T01:42:41.161Z · 计划修订 7
+采用确认时间：2026-10-14T02:07:21.727Z · 计划修订 11
 采用参数
 值
 来源
@@ -133,12 +133,12 @@
 示例母液取液量
 10 µL
 计算后确认
-示例母液取液量 · dilution dilution-v2 · 确认 2026-10-14T01:42:41.161Z
+示例母液取液量 · dilution dilution-v2 · 确认 2026-10-14T02:07:21.727Z
 输入：{"mode":"final","finalVolume":100,"finalVolumeUnit":"µL","stockConcentration":100,"targetConcentration":10,"stockConcentrationUnit":"µM","targetConcentrationUnit":"µM"}
 当时计算结果：10 µL
 体积可加和近似 / Assumes additive volumes.
 共同准备：核对标签和记录编号。
-SYN-b9e2edc6-3b62-4995-b77d-4c0d11eccccd · 350／600 µL 合成规程 · v1.0
+SYN-79b5ab5c-dbd4-464b-a250-d996a01b0b48 · 350／600 µL 合成规程 · v1.0
 ✓ 核对样本
 标记管号
 确认原始记录时间
@@ -148,7 +148,7 @@
 记录时间
 实际 Proteinase K
 50 µL
-2026-10-14T01:42:47.535Z
+2026-10-14T02:07:30.015Z
 组分
 用量
 Proteinase K
@@ -162,7 +162,7 @@
 独立稀释示例取母液 10 µL；这是软件测试，不是试剂方案的附加用量。
 未完成 孵育
 孵育 10 min，计时结束后仍需人工确认。
-高脂样本补充处理 · 不适用于本次实验（来源 cmv7g3ccr0007w6os2aa9gaf3:lipid）</t>
+高脂样本补充处理 · 不适用于本次实验（来源 cmv7gz2j200078fosfu1bvjzs:lipid）</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
docs: attach final release-container and cross-timezone evidence
</commit_message>
<xml_diff>
--- a/docs/structured-protocol/20261014/evidence/experiment.xlsx
+++ b/docs/structured-protocol/20261014/evidence/experiment.xlsx
@@ -76,13 +76,13 @@
     <t>tags</t>
   </si>
   <si>
-    <t>合成体系验收 79b5ab5c-dbd4-464b-a250-d996a01b0b48</t>
-  </si>
-  <si>
-    <t>SYN-79b5ab5c-dbd4-464b-a250-d996a01b0b48</t>
-  </si>
-  <si>
-    <t>EXP-056</t>
+    <t>合成体系验收 88d664d2-3767-48f0-a72d-454ea4e871cc</t>
+  </si>
+  <si>
+    <t>SYN-88d664d2-3767-48f0-a72d-454ea4e871cc</t>
+  </si>
+  <si>
+    <t>EXP-067</t>
   </si>
   <si>
     <t>合成验收 · 页面创建与执行</t>
@@ -106,9 +106,9 @@
     <t>350／600 µL 合成规程 · 1.0</t>
   </si>
   <si>
-    <t>本次执行记录 · 当前实验组 · 源版本 350／600 µL 合成规程 v1.0（cmv7gz2j200078fosfu1bvjzs）
+    <t>本次执行记录 · 当前实验组 · 源版本 350／600 µL 合成规程 v1.0（cmv7hc31z0007doosss2xfg0a）
 裂解体积：350 µL；样本性质：普通样本
-采用确认时间：2026-10-14T02:07:21.727Z · 计划修订 11
+采用确认时间：2026-10-14T02:17:28.042Z · 计划修订 11
 采用参数
 值
 来源
@@ -133,12 +133,12 @@
 示例母液取液量
 10 µL
 计算后确认
-示例母液取液量 · dilution dilution-v2 · 确认 2026-10-14T02:07:21.727Z
+示例母液取液量 · dilution dilution-v2 · 确认 2026-10-14T02:17:28.042Z
 输入：{"mode":"final","finalVolume":100,"finalVolumeUnit":"µL","stockConcentration":100,"targetConcentration":10,"stockConcentrationUnit":"µM","targetConcentrationUnit":"µM"}
 当时计算结果：10 µL
 体积可加和近似 / Assumes additive volumes.
 共同准备：核对标签和记录编号。
-SYN-79b5ab5c-dbd4-464b-a250-d996a01b0b48 · 350／600 µL 合成规程 · v1.0
+SYN-88d664d2-3767-48f0-a72d-454ea4e871cc · 350／600 µL 合成规程 · v1.0
 ✓ 核对样本
 标记管号
 确认原始记录时间
@@ -148,7 +148,7 @@
 记录时间
 实际 Proteinase K
 50 µL
-2026-10-14T02:07:30.015Z
+2026-10-14T02:17:36.480Z
 组分
 用量
 Proteinase K
@@ -162,7 +162,7 @@
 独立稀释示例取母液 10 µL；这是软件测试，不是试剂方案的附加用量。
 未完成 孵育
 孵育 10 min，计时结束后仍需人工确认。
-高脂样本补充处理 · 不适用于本次实验（来源 cmv7gz2j200078fosfu1bvjzs:lipid）</t>
+高脂样本补充处理 · 不适用于本次实验（来源 cmv7hc31z0007doosss2xfg0a:lipid）</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
docs: record final protocol follow-up acceptance and physical limits
</commit_message>
<xml_diff>
--- a/docs/structured-protocol/20261014/evidence/experiment.xlsx
+++ b/docs/structured-protocol/20261014/evidence/experiment.xlsx
@@ -76,13 +76,13 @@
     <t>tags</t>
   </si>
   <si>
-    <t>合成体系验收 88d664d2-3767-48f0-a72d-454ea4e871cc</t>
-  </si>
-  <si>
-    <t>SYN-88d664d2-3767-48f0-a72d-454ea4e871cc</t>
-  </si>
-  <si>
-    <t>EXP-067</t>
+    <t>合成体系验收 a6dfc410-c299-44fc-b93b-652f764e1054</t>
+  </si>
+  <si>
+    <t>SYN-a6dfc410-c299-44fc-b93b-652f764e1054</t>
+  </si>
+  <si>
+    <t>EXP-1791968638018</t>
   </si>
   <si>
     <t>合成验收 · 页面创建与执行</t>
@@ -106,9 +106,9 @@
     <t>350／600 µL 合成规程 · 1.0</t>
   </si>
   <si>
-    <t>本次执行记录 · 当前实验组 · 源版本 350／600 µL 合成规程 v1.0（cmv7hc31z0007doosss2xfg0a）
+    <t>本次执行记录 · 当前实验组 · 源版本 350／600 µL 合成规程 v1.0（cmv7wm0hb0007b5oslcm9zkzw）
 裂解体积：350 µL；样本性质：普通样本
-采用确认时间：2026-10-14T02:17:28.042Z · 计划修订 11
+采用确认时间：2026-10-14T09:25:07.010Z · 计划修订 11
 采用参数
 值
 来源
@@ -133,12 +133,12 @@
 示例母液取液量
 10 µL
 计算后确认
-示例母液取液量 · dilution dilution-v2 · 确认 2026-10-14T02:17:28.042Z
+示例母液取液量 · dilution dilution-v2 · 确认 2026-10-14T09:25:07.010Z
 输入：{"mode":"final","finalVolume":100,"finalVolumeUnit":"µL","stockConcentration":100,"targetConcentration":10,"stockConcentrationUnit":"µM","targetConcentrationUnit":"µM"}
 当时计算结果：10 µL
 体积可加和近似 / Assumes additive volumes.
 共同准备：核对标签和记录编号。
-SYN-88d664d2-3767-48f0-a72d-454ea4e871cc · 350／600 µL 合成规程 · v1.0
+SYN-a6dfc410-c299-44fc-b93b-652f764e1054 · 350／600 µL 合成规程 · v1.0
 ✓ 核对样本
 标记管号
 确认原始记录时间
@@ -148,7 +148,7 @@
 记录时间
 实际 Proteinase K
 50 µL
-2026-10-14T02:17:36.480Z
+2026-10-14T09:25:15.683Z
 组分
 用量
 Proteinase K
@@ -162,7 +162,7 @@
 独立稀释示例取母液 10 µL；这是软件测试，不是试剂方案的附加用量。
 未完成 孵育
 孵育 10 min，计时结束后仍需人工确认。
-高脂样本补充处理 · 不适用于本次实验（来源 cmv7hc31z0007doosss2xfg0a:lipid）</t>
+高脂样本补充处理 · 不适用于本次实验（来源 cmv7wm0hb0007b5oslcm9zkzw:lipid）</t>
   </si>
 </sst>
 </file>

</xml_diff>